<commit_message>
Updated docs for accuracy and clarity
</commit_message>
<xml_diff>
--- a/Analysis Examples/Unposted-GL-Batch-Analysis.xlsx
+++ b/Analysis Examples/Unposted-GL-Batch-Analysis.xlsx
@@ -6,11 +6,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GL Batch Analysis" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysis" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unposted GL Batches" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Unposted GL Batches'!$A$2:$M$2</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Analysis'!$A$1:$R$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Unposted GL Batches'!$A$2:$M$19</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="23">
+  <fonts count="39">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -145,8 +146,101 @@
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00404040"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="008B0000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="006B3A00"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="004A3B00"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="008B0000"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="006B3A00"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="004A3B00"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="26">
     <fill>
       <patternFill/>
     </fill>
@@ -233,6 +327,54 @@
         <fgColor rgb="FFF5DEB3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+        <bgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0E0"/>
+        <bgColor rgb="00FFE0E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF0DC"/>
+        <bgColor rgb="00FFF0DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEFBD8"/>
+        <bgColor rgb="00FEFBD8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5DEB3"/>
+        <bgColor rgb="00F5DEB3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -273,7 +415,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -481,6 +623,97 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -570,7 +803,7 @@
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>30</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -607,20 +840,13 @@
               </a:solidFill>
               <a:latin typeface="Arial"/>
             </a:rPr>
-            <a:t>Unposted GL Batch Analysis</a:t>
+            <a:t>Unposted GL Batches Analysis</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr algn="l">
-            <a:spcBef>
-              <a:spcPts val="400"/>
-            </a:spcBef>
-          </a:pPr>
+          <a:pPr algn="l"/>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
               <a:latin typeface="Arial"/>
             </a:rPr>
             <a:t> </a:t>
@@ -639,7 +865,7 @@
               </a:solidFill>
               <a:latin typeface="Arial"/>
             </a:rPr>
-            <a:t>What is an Unposted GL Batch?</a:t>
+            <a:t>What is an unposted GL batch?</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -651,20 +877,13 @@
               </a:solidFill>
               <a:latin typeface="Arial"/>
             </a:rPr>
-            <a:t>In JD Edwards, GL transactions are grouped into batches before posting to account balances (F0902). An unposted batch means transactions exist in the GL detail table (F0911) but have not been summarized — invisible to period-end reporting.</a:t>
+            <a:t>Every JD Edwards GL transaction passes through two gates: approval, then posting (R09801). Until both gates clear, the transaction exists in F0911 but isn't reflected in F0902 account balances. RapidReconciler reports the gap as GL Batches variance.</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr algn="l">
-            <a:spcBef>
-              <a:spcPts val="400"/>
-            </a:spcBef>
-          </a:pPr>
+          <a:pPr algn="l"/>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
               <a:latin typeface="Arial"/>
             </a:rPr>
             <a:t> </a:t>
@@ -695,20 +914,13 @@
               </a:solidFill>
               <a:latin typeface="Arial"/>
             </a:rPr>
-            <a:t>Unposted batches create the GL Batches variance in RapidReconciler. The variance must reach zero before period close — any open batch means the financial statements do not reflect all activity.</a:t>
+            <a:t>The GL Batches variance must be $0 before period-end close. A non-zero balance means F0902 doesn't reflect all posted activity, and any closing journal entries calculated against those balances will be on an incomplete picture.</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr algn="l">
-            <a:spcBef>
-              <a:spcPts val="400"/>
-            </a:spcBef>
-          </a:pPr>
+          <a:pPr algn="l"/>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
               <a:latin typeface="Arial"/>
             </a:rPr>
             <a:t> </a:t>
@@ -739,20 +951,13 @@
               </a:solidFill>
               <a:latin typeface="Arial"/>
             </a:rPr>
-            <a:t>Three priority levels: batches stuck In Use (require a manual status reset), batches pending approval (require supervisor sign-off), and approved batches awaiting the next posting run.</a:t>
+            <a:t>An at-a-glance Issue Summary table partitioning the unposted batches by status combination, one Finding card per pattern (Scope, Pattern, Resolution), and an Action Plan in execution order.</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr algn="l">
-            <a:spcBef>
-              <a:spcPts val="400"/>
-            </a:spcBef>
-          </a:pPr>
+          <a:pPr algn="l"/>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
               <a:latin typeface="Arial"/>
             </a:rPr>
             <a:t> </a:t>
@@ -783,7 +988,7 @@
               </a:solidFill>
               <a:latin typeface="Arial"/>
             </a:rPr>
-            <a:t>GL Batch Analysis = findings and recommended actions. Unposted GL Batches = source export data.</a:t>
+            <a:t>Analysis sheet = findings and actions.   Unposted GL Batches sheet = full source export with AutoFilter on the header row — filter on Approval_Status, Posting_Status, or Type to drill into a specific finding.</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -1080,793 +1285,722 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" style="29" min="1" max="1"/>
-    <col width="80" customWidth="1" style="29" min="2" max="2"/>
-    <col width="30" customWidth="1" style="29" min="3" max="3"/>
-    <col width="8" customWidth="1" style="29" min="6" max="6"/>
+    <col width="24" customWidth="1" style="29" min="1" max="1"/>
+    <col width="30" customWidth="1" style="29" min="2" max="2"/>
+    <col width="38" customWidth="1" style="29" min="3" max="3"/>
+    <col width="22" customWidth="1" style="29" min="4" max="4"/>
+    <col width="22" customWidth="1" style="29" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" s="29">
-      <c r="A1" s="40" t="inlineStr">
-        <is>
-          <t>RapidReconciler — GL Batch Analysis</t>
-        </is>
-      </c>
-      <c r="F1" s="75" t="n"/>
-    </row>
-    <row r="2" s="29">
-      <c r="A2" s="41" t="n"/>
-      <c r="B2" s="41" t="n"/>
-      <c r="C2" s="41" t="n"/>
-      <c r="F2" s="76" t="n"/>
-    </row>
-    <row r="3" s="29">
-      <c r="A3" s="42" t="inlineStr">
-        <is>
-          <t>REPORT SUMMARY</t>
-        </is>
-      </c>
-      <c r="F3" s="77" t="n"/>
-    </row>
-    <row r="4" ht="42" customHeight="1" s="29">
-      <c r="A4" s="43" t="inlineStr">
-        <is>
-          <t>Report</t>
-        </is>
-      </c>
-      <c r="B4" s="24" t="inlineStr">
+    <row r="1" ht="6" customHeight="1" s="29">
+      <c r="A1" s="78" t="n"/>
+      <c r="B1" s="78" t="n"/>
+      <c r="C1" s="78" t="n"/>
+      <c r="D1" s="78" t="n"/>
+      <c r="E1" s="78" t="n"/>
+    </row>
+    <row r="2" ht="38" customHeight="1" s="29">
+      <c r="A2" s="79" t="inlineStr">
         <is>
           <t>Unposted GL Batches — Period Ending March 31, 2026</t>
         </is>
       </c>
-      <c r="C4" s="41" t="n"/>
-      <c r="F4" s="76" t="n"/>
-    </row>
-    <row r="5" s="29">
-      <c r="A5" s="43" t="inlineStr">
-        <is>
-          <t>Generated</t>
-        </is>
-      </c>
-      <c r="B5" s="24" t="inlineStr">
-        <is>
-          <t>Wednesday, April 22, 2026  08:31 AM</t>
-        </is>
-      </c>
-      <c r="C5" s="41" t="n"/>
-      <c r="F5" s="76" t="n"/>
-    </row>
-    <row r="6" s="29">
-      <c r="A6" s="43" t="inlineStr">
-        <is>
-          <t>Total Records</t>
-        </is>
-      </c>
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>17 rows across 16 distinct batches</t>
-        </is>
-      </c>
-      <c r="C6" s="41" t="n"/>
-      <c r="F6" s="77" t="n"/>
-    </row>
-    <row r="7" ht="42" customHeight="1" s="29">
-      <c r="A7" s="43" t="inlineStr">
-        <is>
-          <t>Total Variance</t>
-        </is>
-      </c>
-      <c r="B7" s="62" t="inlineStr">
-        <is>
-          <t>$162,174.95</t>
-        </is>
-      </c>
-      <c r="C7" s="41" t="n"/>
-      <c r="F7" s="76" t="n"/>
-    </row>
-    <row r="8" s="29">
-      <c r="A8" s="43" t="inlineStr">
-        <is>
-          <t>Companies</t>
-        </is>
-      </c>
-      <c r="B8" s="24" t="inlineStr">
-        <is>
-          <t>00010, 00030, 00070, 00080, 00090</t>
-        </is>
-      </c>
-      <c r="C8" s="41" t="n"/>
-      <c r="F8" s="76" t="n"/>
-    </row>
-    <row r="9" s="29">
-      <c r="A9" s="43" t="inlineStr">
-        <is>
-          <t>Batch Types</t>
-        </is>
-      </c>
-      <c r="B9" s="24" t="inlineStr">
-        <is>
-          <t>G (General Journal), IB (Inventory Balance), N (Inventory), O (PO Receipts), V (Voucher)</t>
-        </is>
-      </c>
-      <c r="C9" s="41" t="n"/>
-      <c r="F9" s="77" t="n"/>
-    </row>
-    <row r="10" ht="42" customHeight="1" s="29">
-      <c r="A10" s="41" t="n"/>
-      <c r="B10" s="41" t="n"/>
-      <c r="C10" s="41" t="n"/>
-      <c r="F10" s="76" t="n"/>
-    </row>
-    <row r="11" s="29">
-      <c r="A11" s="42" t="inlineStr">
-        <is>
-          <t>STATUS SUMMARY</t>
-        </is>
-      </c>
-      <c r="F11" s="76" t="n"/>
-    </row>
-    <row r="12" s="29">
-      <c r="A12" s="45" t="inlineStr">
-        <is>
-          <t>Status Combination</t>
-        </is>
-      </c>
-      <c r="B12" s="45" t="inlineStr">
-        <is>
-          <t>Rows / Batches</t>
-        </is>
-      </c>
-      <c r="C12" s="45" t="inlineStr">
+    </row>
+    <row r="3" ht="24" customHeight="1" s="29">
+      <c r="A3" s="80" t="inlineStr">
+        <is>
+          <t>$162,174.95 unposted across 16 batches — 5 findings across 5 companies, 17 rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="29">
+      <c r="A4" s="81" t="inlineStr">
+        <is>
+          <t>Generated  April 25, 2026          Companies  10, 30, 70, 80, 90          Batch Types  G, IB, N, O, V          Distinct Batches  16</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="12" customHeight="1" s="29"/>
+    <row r="6" ht="28" customHeight="1" s="29">
+      <c r="A6" s="82" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="B6" s="82" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="C6" s="82" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="D6" s="83" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="F12" s="77" t="n"/>
-    </row>
-    <row r="13" ht="42" customHeight="1" s="29">
-      <c r="A13" s="63" t="inlineStr">
-        <is>
-          <t>Pending Approval / In Use</t>
-        </is>
-      </c>
-      <c r="B13" s="63" t="inlineStr">
-        <is>
-          <t>5 rows — 5 batches (Co 00080, Type O)</t>
-        </is>
-      </c>
-      <c r="C13" s="63" t="inlineStr">
+      <c r="E6" s="83" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1" s="29">
+      <c r="A7" s="84" t="inlineStr">
+        <is>
+          <t>"In Use" stuck batches — manual P0011 reset required</t>
+        </is>
+      </c>
+      <c r="B7" s="85" t="inlineStr">
+        <is>
+          <t>Co 80, Type O</t>
+        </is>
+      </c>
+      <c r="C7" s="85" t="inlineStr">
+        <is>
+          <t>5 batches · oldest 29d · scheduler user SCHED01</t>
+        </is>
+      </c>
+      <c r="D7" s="86" t="inlineStr">
         <is>
           <t>$156,598.12</t>
         </is>
       </c>
-      <c r="F13" s="76" t="n"/>
-    </row>
-    <row r="14" ht="28" customHeight="1" s="29">
-      <c r="A14" s="64" t="inlineStr">
-        <is>
-          <t>Pending Approval / Pending</t>
-        </is>
-      </c>
-      <c r="B14" s="64" t="inlineStr">
-        <is>
-          <t>4 rows — 10 batches (Co 00090 IB, Co 00070 G, Co 00030 V)</t>
-        </is>
-      </c>
-      <c r="C14" s="64" t="inlineStr">
-        <is>
-          <t>$7,003.27</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1" s="29">
-      <c r="A15" s="65" t="inlineStr">
-        <is>
-          <t>Approved / Approved (unposted)</t>
-        </is>
-      </c>
-      <c r="B15" s="65" t="inlineStr">
-        <is>
-          <t>8 rows — 8 batches (Co 00010, Type N)</t>
-        </is>
-      </c>
-      <c r="C15" s="65" t="inlineStr">
+      <c r="E7" s="87" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1" s="29">
+      <c r="A8" s="88" t="inlineStr">
+        <is>
+          <t>Pending — AP voucher needs invoice verification</t>
+        </is>
+      </c>
+      <c r="B8" s="89" t="inlineStr">
+        <is>
+          <t>Co 30, Type V</t>
+        </is>
+      </c>
+      <c r="C8" s="89" t="inlineStr">
+        <is>
+          <t>1 batch (USER04) · age 1d</t>
+        </is>
+      </c>
+      <c r="D8" s="90" t="inlineStr">
+        <is>
+          <t>$13,354.12</t>
+        </is>
+      </c>
+      <c r="E8" s="91" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1" s="29">
+      <c r="A9" s="84" t="inlineStr">
+        <is>
+          <t>Pending — IB batch spanning two accounts</t>
+        </is>
+      </c>
+      <c r="B9" s="85" t="inlineStr">
+        <is>
+          <t>Co 90, Type IB</t>
+        </is>
+      </c>
+      <c r="C9" s="85" t="inlineStr">
+        <is>
+          <t>1 batch (2 rows, both must be approved together) · age 13d</t>
+        </is>
+      </c>
+      <c r="D9" s="86" t="inlineStr">
+        <is>
+          <t>$-5,583.45</t>
+        </is>
+      </c>
+      <c r="E9" s="91" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1" s="29">
+      <c r="A10" s="88" t="inlineStr">
+        <is>
+          <t>Pending — Manual journal entry needs supervisor sign-off</t>
+        </is>
+      </c>
+      <c r="B10" s="89" t="inlineStr">
+        <is>
+          <t>Co 70, Type G</t>
+        </is>
+      </c>
+      <c r="C10" s="89" t="inlineStr">
+        <is>
+          <t>1 batch (USER02) · age 4d</t>
+        </is>
+      </c>
+      <c r="D10" s="90" t="inlineStr">
+        <is>
+          <t>$-767.40</t>
+        </is>
+      </c>
+      <c r="E10" s="91" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1" s="29">
+      <c r="A11" s="84" t="inlineStr">
+        <is>
+          <t>Approved — N-type inventory batches awaiting R09801</t>
+        </is>
+      </c>
+      <c r="B11" s="85" t="inlineStr">
+        <is>
+          <t>Co 10, Type N</t>
+        </is>
+      </c>
+      <c r="C11" s="85" t="inlineStr">
+        <is>
+          <t>8 batches (USER03) · ages 0-1d · routine</t>
+        </is>
+      </c>
+      <c r="D11" s="86" t="inlineStr">
         <is>
           <t>$-1,426.44</t>
         </is>
       </c>
-    </row>
-    <row r="16" s="29">
-      <c r="A16" s="41" t="n"/>
-      <c r="B16" s="41" t="n"/>
-      <c r="C16" s="41" t="n"/>
-    </row>
-    <row r="17" ht="16" customHeight="1" s="29">
-      <c r="A17" s="42" t="inlineStr">
-        <is>
-          <t>FINDINGS BY PRIORITY</t>
-        </is>
-      </c>
-    </row>
+      <c r="E11" s="92" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="14" customHeight="1" s="29"/>
+    <row r="13" ht="28" customHeight="1" s="29">
+      <c r="A13" s="93" t="inlineStr">
+        <is>
+          <t>FINDING 1 — "In Use" posting status — manual P0011 reset required (5 batches)    [Priority 1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="64" customHeight="1" s="29">
+      <c r="A14" s="94" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B14" s="95" t="inlineStr">
+        <is>
+          <t>Company 00080, Type O (Purchase Order Receipts).  5 batches all created by scheduler user SCHED01.  Posting status "In Use" prevents normal posting and will not clear automatically.  Oldest batch is 29 days old; newest is 6 days.  All five point to account 80010.3810.</t>
+        </is>
+      </c>
+      <c r="C14" s="96" t="n"/>
+      <c r="D14" s="96" t="n"/>
+      <c r="E14" s="96" t="n"/>
+    </row>
+    <row r="15" ht="240" customHeight="1" s="29">
+      <c r="A15" s="97" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="B15" s="98" t="inlineStr">
+        <is>
+          <t>RapidReconciler displays "In Use" when the batch posting status in F0011 is in a state that prevents posting — typically because a posting job was interrupted mid-run, leaving the status non-blank but not posted.  This does not mean another user has the batch locked.
+Because the batches come from SCHED01 (a system scheduler) and span 23 days from oldest to newest, the same failure has been recurring silently — no user is monitoring the scheduler output.  This is a systemic issue with the receipt posting job, not a one-time event.
+Affected batches:
+  •  Batch 7000001  (2026-03-02, age 29d)  $171.40
+  •  Batch 7000002  (2026-03-04, age 27d)  $31,688.98
+  •  Batch 7000004  (2026-03-23, age 8d)  $818.42
+  •  Batch 7000005  (2026-03-25, age 6d)  $438.04
+  •  Batch 7000006  (2026-03-25, age 6d)  $123,481.28</t>
+        </is>
+      </c>
+      <c r="C15" s="99" t="n"/>
+      <c r="D15" s="99" t="n"/>
+      <c r="E15" s="99" t="n"/>
+    </row>
+    <row r="16" ht="160" customHeight="1" s="29">
+      <c r="A16" s="94" t="inlineStr">
+        <is>
+          <t>Resolution</t>
+        </is>
+      </c>
+      <c r="B16" s="95" t="inlineStr">
+        <is>
+          <t>Step 1.  Open Batch Header Revisions (P0011) in JD Edwards for each of the five batches above.  For each batch, manually set the posting status back to blank (unposted).
+Step 2.  Approve each batch (the approval status is also currently "Pending approval").  Then run R09801 to post.
+Step 3.  Engage IT to investigate why the SCHED01 receipt-posting job has been failing.  Configure alerting so future occurrences surface immediately rather than accumulating across periods.
+Step 4.  After all five batches are posted, refresh RapidReconciler and confirm Co 80 GL Batches variance has decreased by $156,598.12.</t>
+        </is>
+      </c>
+      <c r="C16" s="96" t="n"/>
+      <c r="D16" s="96" t="n"/>
+      <c r="E16" s="96" t="n"/>
+    </row>
+    <row r="17" ht="10" customHeight="1" s="29"/>
     <row r="18" ht="28" customHeight="1" s="29">
-      <c r="A18" s="63" t="inlineStr">
-        <is>
-          <t>PRIORITY 1 — Immediate Action Required</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1" s="29">
-      <c r="A19" s="45" t="inlineStr">
-        <is>
-          <t>Batch</t>
-        </is>
-      </c>
-      <c r="B19" s="45" t="inlineStr">
-        <is>
-          <t>Detail</t>
-        </is>
-      </c>
-      <c r="C19" s="45" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="28" customHeight="1" s="29">
-      <c r="A20" s="49" t="inlineStr">
-        <is>
-          <t>7000001</t>
-        </is>
-      </c>
-      <c r="B20" s="50" t="inlineStr">
-        <is>
-          <t>Co 00080 | Type O | 2026-03-02 | User: SCHED01 | 29 days before period end</t>
-        </is>
-      </c>
-      <c r="C20" s="49" t="inlineStr">
-        <is>
-          <t>$171.40</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="28" customHeight="1" s="29">
-      <c r="A21" s="49" t="inlineStr">
-        <is>
-          <t>7000002</t>
-        </is>
-      </c>
-      <c r="B21" s="50" t="inlineStr">
-        <is>
-          <t>Co 00080 | Type O | 2026-03-04 | User: SCHED01 | 27 days before period end</t>
-        </is>
-      </c>
-      <c r="C21" s="49" t="inlineStr">
-        <is>
-          <t>$31,688.98</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="28" customHeight="1" s="29">
-      <c r="A22" s="49" t="inlineStr">
-        <is>
-          <t>7000004</t>
-        </is>
-      </c>
-      <c r="B22" s="50" t="inlineStr">
-        <is>
-          <t>Co 00080 | Type O | 2026-03-23 | User: SCHED01 | 8 days before period end</t>
-        </is>
-      </c>
-      <c r="C22" s="49" t="inlineStr">
-        <is>
-          <t>$818.42</t>
-        </is>
-      </c>
-    </row>
+      <c r="A18" s="100" t="inlineStr">
+        <is>
+          <t>FINDING 2 — IB batch spanning two accounts — multi-account approval required    [Priority 2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="96" customHeight="1" s="29">
+      <c r="A19" s="94" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B19" s="95" t="inlineStr">
+        <is>
+          <t>Company 00090, Type IB (Inventory Balance Adjustments).  Batch 7000003 from USER01, dated 2026-03-18 (age 13 days).  2 rows totalling $-5,583.45 across two accounts.
+  •  Account 90010.3810  $-2,232.75
+  •  Account 90040.3810  $-3,350.70</t>
+        </is>
+      </c>
+      <c r="C19" s="96" t="n"/>
+      <c r="D19" s="96" t="n"/>
+      <c r="E19" s="96" t="n"/>
+    </row>
+    <row r="20" ht="112" customHeight="1" s="29">
+      <c r="A20" s="97" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="B20" s="98" t="inlineStr">
+        <is>
+          <t>An IB batch is created when an inventory balance adjustment affects multiple accounts — for example, a cost change that posts across two business units.  Both rows share batch number 7000003 and must be reviewed and approved together; approving the batch clears both rows simultaneously.
+13 days old is meaningful — IB batches from cost changes are typically approved within a day or two by inventory accounting.  Worth confirming with USER01 why this one has been waiting.</t>
+        </is>
+      </c>
+      <c r="C20" s="99" t="n"/>
+      <c r="D20" s="99" t="n"/>
+      <c r="E20" s="99" t="n"/>
+    </row>
+    <row r="21" ht="160" customHeight="1" s="29">
+      <c r="A21" s="94" t="inlineStr">
+        <is>
+          <t>Resolution</t>
+        </is>
+      </c>
+      <c r="B21" s="95" t="inlineStr">
+        <is>
+          <t>Step 1.  Navigate to P0011 and locate batch 7000003.  Review both account entries to confirm the amounts and accounts are correct.  Verify the entries offset each other or otherwise represent a coherent inventory balance adjustment.
+Step 2.  If the entries do not appear to offset or the accounts are unexpected, contact USER01 before approving.  Do not approve a batch that doesn't make accounting sense.
+Step 3.  Once verified, approve the batch.  Both rows clear simultaneously since they share the batch number.
+Step 4.  Run R09801 to post.</t>
+        </is>
+      </c>
+      <c r="C21" s="96" t="n"/>
+      <c r="D21" s="96" t="n"/>
+      <c r="E21" s="96" t="n"/>
+    </row>
+    <row r="22" ht="10" customHeight="1" s="29"/>
     <row r="23" ht="28" customHeight="1" s="29">
-      <c r="A23" s="49" t="inlineStr">
-        <is>
-          <t>7000005</t>
-        </is>
-      </c>
-      <c r="B23" s="50" t="inlineStr">
-        <is>
-          <t>Co 00080 | Type O | 2026-03-25 | User: SCHED01 | 6 days before period end</t>
-        </is>
-      </c>
-      <c r="C23" s="49" t="inlineStr">
-        <is>
-          <t>$438.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="28" customHeight="1" s="29">
-      <c r="A24" s="49" t="inlineStr">
-        <is>
-          <t>7000006</t>
-        </is>
-      </c>
-      <c r="B24" s="50" t="inlineStr">
-        <is>
-          <t>Co 00080 | Type O | 2026-03-25 | User: SCHED01 | 6 days before period end</t>
-        </is>
-      </c>
-      <c r="C24" s="49" t="inlineStr">
-        <is>
-          <t>$123,481.28</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="16" customHeight="1" s="29">
-      <c r="A25" s="49" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B25" s="51" t="n"/>
-      <c r="C25" s="49" t="inlineStr">
-        <is>
-          <t>$156,598.12</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="75" customHeight="1" s="29">
-      <c r="A26" s="66" t="inlineStr">
-        <is>
-          <t>Posting Status = "In Use" on O-type batches requires a manual status reset in JD Edwards. Open each batch in the Batch Header Revisions screen (P0011), locate the batch by number, and set the posting status back to blank (unposted). The oldest batch (7000001) is 29 days old. All five are from user SCHED01 (system scheduler), suggesting a recurring posting job interruption on PO receipt processing in Co 00080. Resolution: Open P0011 for each batch, reset posting status to blank, approve, then run R09801. Engage IT to investigate why the scheduler posting is being interrupted and configure alerting to prevent future accumulation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="16" customHeight="1" s="29">
-      <c r="A27" s="41" t="n"/>
-      <c r="B27" s="41" t="n"/>
-      <c r="C27" s="41" t="n"/>
-    </row>
+      <c r="A23" s="100" t="inlineStr">
+        <is>
+          <t>FINDING 3 — Manual journal entry — supervisor sign-off required    [Priority 2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1" s="29">
+      <c r="A24" s="94" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B24" s="95" t="inlineStr">
+        <is>
+          <t>Company 00070, Type G (General Journal).  Batch 7000007 from USER02, dated 2026-03-27 (age 4 days).  Account 70.3810, $-767.40.</t>
+        </is>
+      </c>
+      <c r="C24" s="96" t="n"/>
+      <c r="D24" s="96" t="n"/>
+      <c r="E24" s="96" t="n"/>
+    </row>
+    <row r="25" ht="112" customHeight="1" s="29">
+      <c r="A25" s="97" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="B25" s="98" t="inlineStr">
+        <is>
+          <t>G-type batches are manual journal entries created in P0911.  They typically require manual approval — and per most segregation-of-duties policies, the approver must be a different person from the user who entered the batch.  Until an authorized approver reviews and approves it, the batch will not post.
+At 4 days old this is not yet escalation territory, but a manual journal entry sitting unposted across a period end can affect closing balances.  The guide flags 5 business days as the escalation threshold.</t>
+        </is>
+      </c>
+      <c r="C25" s="99" t="n"/>
+      <c r="D25" s="99" t="n"/>
+      <c r="E25" s="99" t="n"/>
+    </row>
+    <row r="26" ht="176" customHeight="1" s="29">
+      <c r="A26" s="94" t="inlineStr">
+        <is>
+          <t>Resolution</t>
+        </is>
+      </c>
+      <c r="B26" s="95" t="inlineStr">
+        <is>
+          <t>Step 1.  Contact USER02 to confirm the purpose of the journal entry.  Manual entries should have a clear business reason documented.
+Step 2.  Obtain supervisor sign-off per segregation-of-duties policy.  The supervisor should not be USER02.
+Step 3.  Approve in P0011.
+Step 4.  Run R09801 to post.
+Step 5.  If USER02 cannot be contacted within 1 business day, escalate to the finance manager — the batch will exceed the 5-business-day escalation threshold soon.</t>
+        </is>
+      </c>
+      <c r="C26" s="96" t="n"/>
+      <c r="D26" s="96" t="n"/>
+      <c r="E26" s="96" t="n"/>
+    </row>
+    <row r="27" ht="10" customHeight="1" s="29"/>
     <row r="28" ht="28" customHeight="1" s="29">
-      <c r="A28" s="64" t="inlineStr">
-        <is>
-          <t>PRIORITY 10 — Approval Required</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="16" customHeight="1" s="29">
-      <c r="A29" s="45" t="inlineStr">
-        <is>
-          <t>Batch</t>
-        </is>
-      </c>
-      <c r="B29" s="45" t="inlineStr">
-        <is>
-          <t>Detail</t>
-        </is>
-      </c>
-      <c r="C29" s="45" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="28" customHeight="1" s="29">
-      <c r="A30" s="67" t="inlineStr">
-        <is>
-          <t>7000003</t>
-        </is>
-      </c>
-      <c r="B30" s="68" t="inlineStr">
-        <is>
-          <t>Co 00090 | Type IB | 2026-03-18 | User: USER01 | 10 account lines: $-10,232.75 + $-3,350.70</t>
-        </is>
-      </c>
-      <c r="C30" s="67" t="inlineStr">
-        <is>
-          <t>$-5,583.45</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="28" customHeight="1" s="29">
-      <c r="A31" s="67" t="inlineStr">
-        <is>
-          <t>7000007</t>
-        </is>
-      </c>
-      <c r="B31" s="68" t="inlineStr">
-        <is>
-          <t>Co 00070 | Type G  | 2026-03-27 | User: USER02 | Manual journal entry — 4 days old</t>
-        </is>
-      </c>
-      <c r="C31" s="67" t="inlineStr">
-        <is>
-          <t>$-767.40</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="28" customHeight="1" s="29">
-      <c r="A32" s="67" t="inlineStr">
-        <is>
-          <t>7000008</t>
-        </is>
-      </c>
-      <c r="B32" s="68" t="inlineStr">
-        <is>
-          <t>Co 00030 | Type V  | 2026-03-30 | User: USER04 | AP voucher — 1 day old</t>
-        </is>
-      </c>
-      <c r="C32" s="67" t="inlineStr">
-        <is>
-          <t>$13,354.12</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="16" customHeight="1" s="29">
-      <c r="A33" s="67" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B33" s="69" t="n"/>
-      <c r="C33" s="67" t="inlineStr">
-        <is>
-          <t>$7,003.27</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="75" customHeight="1" s="29">
-      <c r="A34" s="66" t="inlineStr">
-        <is>
-          <t>Three batches require manual approval before posting. IB batch 7000003 (USER01) spans two inventory accounts in Co 00090 — both rows must be resolved together. G batch 7000007 (USER02) is a manual journal entry that requires supervisor review per segregation of duties policy. V batch 7000008 (USER04) is an AP voucher in Co 00030 — confirm the invoice is valid before approving. Resolution: Approve each batch in P0011, then run R09801.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="16" customHeight="1" s="29">
-      <c r="A35" s="41" t="n"/>
-      <c r="B35" s="41" t="n"/>
-      <c r="C35" s="41" t="n"/>
-    </row>
-    <row r="36" ht="28" customHeight="1" s="29">
-      <c r="A36" s="65" t="inlineStr">
-        <is>
-          <t>PRIORITY 3 — Post Required (Approved)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="16" customHeight="1" s="29">
-      <c r="A37" s="45" t="inlineStr">
-        <is>
-          <t>Batch</t>
-        </is>
-      </c>
-      <c r="B37" s="45" t="inlineStr">
-        <is>
-          <t>Detail</t>
-        </is>
-      </c>
-      <c r="C37" s="45" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="16" customHeight="1" s="29">
-      <c r="A38" s="70" t="inlineStr">
-        <is>
-          <t>7000009</t>
-        </is>
-      </c>
-      <c r="B38" s="70" t="inlineStr">
-        <is>
-          <t>Co 00010 | Type N | 2026-03-30 | User: USER03</t>
-        </is>
-      </c>
-      <c r="C38" s="70" t="inlineStr">
-        <is>
-          <t>$-33.88</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="16" customHeight="1" s="29">
-      <c r="A39" s="70" t="inlineStr">
-        <is>
-          <t>7000010</t>
-        </is>
-      </c>
-      <c r="B39" s="70" t="inlineStr">
-        <is>
-          <t>Co 00010 | Type N | 2026-03-30 | User: USER03</t>
-        </is>
-      </c>
-      <c r="C39" s="70" t="inlineStr">
-        <is>
-          <t>$250.28</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="16" customHeight="1" s="29">
-      <c r="A40" s="70" t="inlineStr">
-        <is>
-          <t>7000011</t>
-        </is>
-      </c>
-      <c r="B40" s="70" t="inlineStr">
-        <is>
-          <t>Co 00010 | Type N | 2026-03-31 | User: USER03</t>
-        </is>
-      </c>
-      <c r="C40" s="70" t="inlineStr">
-        <is>
-          <t>$-97.50</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="16" customHeight="1" s="29">
-      <c r="A41" s="70" t="inlineStr">
-        <is>
-          <t>7000012</t>
-        </is>
-      </c>
-      <c r="B41" s="70" t="inlineStr">
-        <is>
-          <t>Co 00010 | Type N | 2026-03-31 | User: USER03</t>
-        </is>
-      </c>
-      <c r="C41" s="70" t="inlineStr">
-        <is>
-          <t>$-72.37</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="16" customHeight="1" s="29">
-      <c r="A42" s="70" t="inlineStr">
-        <is>
-          <t>7000013</t>
-        </is>
-      </c>
-      <c r="B42" s="70" t="inlineStr">
-        <is>
-          <t>Co 00010 | Type N | 2026-03-31 | User: USER03</t>
-        </is>
-      </c>
-      <c r="C42" s="70" t="inlineStr">
-        <is>
-          <t>$-40.97</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="16" customHeight="1" s="29">
-      <c r="A43" s="70" t="inlineStr">
-        <is>
-          <t>7000014</t>
-        </is>
-      </c>
-      <c r="B43" s="70" t="inlineStr">
-        <is>
-          <t>Co 00010 | Type N | 2026-03-31 | User: USER03</t>
-        </is>
-      </c>
-      <c r="C43" s="70" t="inlineStr">
-        <is>
-          <t>$-157.63</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="16" customHeight="1" s="29">
-      <c r="A44" s="70" t="inlineStr">
-        <is>
-          <t>7000015</t>
-        </is>
-      </c>
-      <c r="B44" s="70" t="inlineStr">
-        <is>
-          <t>Co 00010 | Type N | 2026-03-31 | User: USER03</t>
-        </is>
-      </c>
-      <c r="C44" s="70" t="inlineStr">
-        <is>
-          <t>$-154.36</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="16" customHeight="1" s="29">
-      <c r="A45" s="70" t="inlineStr">
-        <is>
-          <t>7000016</t>
-        </is>
-      </c>
-      <c r="B45" s="70" t="inlineStr">
-        <is>
-          <t>Co 00010 | Type N | 2026-03-31 | User: USER03</t>
-        </is>
-      </c>
-      <c r="C45" s="70" t="inlineStr">
-        <is>
-          <t>$-1,120.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="16" customHeight="1" s="29">
-      <c r="A46" s="71" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B46" s="72" t="n"/>
-      <c r="C46" s="71" t="inlineStr">
-        <is>
-          <t>$-1,426.44</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="75" customHeight="1" s="29">
-      <c r="A47" s="66" t="inlineStr">
-        <is>
-          <t>8 N-type (inventory) batches in Co 00010 from user USER03 are approved but have not been posted. All are dated March 30–31, 2026 (0–1 days before period end). No immediate concern — likely entered on the last day of the period and will be picked up in the next R09801 posting run. Resolution: Run R09801 for Co 00010 to post all approved N-type batches.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="16" customHeight="1" s="29">
-      <c r="A48" s="41" t="n"/>
-      <c r="B48" s="41" t="n"/>
-      <c r="C48" s="41" t="n"/>
-    </row>
-    <row r="49" ht="16" customHeight="1" s="29">
-      <c r="A49" s="42" t="inlineStr">
-        <is>
-          <t>RECOMMENDED ACTIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="16" customHeight="1" s="29">
-      <c r="A50" s="45" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="B50" s="45" t="inlineStr">
+      <c r="A28" s="100" t="inlineStr">
+        <is>
+          <t>FINDING 4 — AP voucher — invoice verification required before approval    [Priority 2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1" s="29">
+      <c r="A29" s="94" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B29" s="95" t="inlineStr">
+        <is>
+          <t>Company 00030, Type V (Accounts Payable Vouchers).  Batch 7000008 from USER04, dated 2026-03-30 (age 1 day).  Account 30.3810, $13,354.12.</t>
+        </is>
+      </c>
+      <c r="C29" s="96" t="n"/>
+      <c r="D29" s="96" t="n"/>
+      <c r="E29" s="96" t="n"/>
+    </row>
+    <row r="30" ht="128" customHeight="1" s="29">
+      <c r="A30" s="97" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="B30" s="98" t="inlineStr">
+        <is>
+          <t>V-type batches are AP vouchers — typically supplier invoices entered through P0411 or matched via P4314.  They require manual approval as part of payment controls.  At 1 day old this is routine — most AP vouchers clear within a normal approval cycle.
+The verification before approving matters: an incorrectly entered voucher that posts to an inventory account would appear later as a GL-only variance in RapidReconciler's Transactions page.  Catching it at the approval gate is much cleaner than fixing it after posting.</t>
+        </is>
+      </c>
+      <c r="C30" s="99" t="n"/>
+      <c r="D30" s="99" t="n"/>
+      <c r="E30" s="99" t="n"/>
+    </row>
+    <row r="31" ht="144" customHeight="1" s="29">
+      <c r="A31" s="94" t="inlineStr">
+        <is>
+          <t>Resolution</t>
+        </is>
+      </c>
+      <c r="B31" s="95" t="inlineStr">
+        <is>
+          <t>Step 1.  Locate the supplier invoice underlying the voucher and verify the amount matches the batch amount.
+Step 2.  Confirm the GL account in the LongAccount column (30.3810) is correct for the purchase.  AP vouchers should not be posting to inventory or balance sheet accounts unless the underlying transaction warrants it.
+Step 3.  Approve in P0011.
+Step 4.  Run R09801 to post.</t>
+        </is>
+      </c>
+      <c r="C31" s="96" t="n"/>
+      <c r="D31" s="96" t="n"/>
+      <c r="E31" s="96" t="n"/>
+    </row>
+    <row r="32" ht="10" customHeight="1" s="29"/>
+    <row r="33" ht="28" customHeight="1" s="29">
+      <c r="A33" s="101" t="inlineStr">
+        <is>
+          <t>FINDING 5 — Approved inventory batches awaiting next posting run (8 batches)    [Priority 3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1" s="29">
+      <c r="A34" s="94" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B34" s="95" t="inlineStr">
+        <is>
+          <t>Company 00010, Type N (Inventory Adjustments / Issues / Transfers).  8 batches all from USER03, dated 2026-03-30, 2026-03-31.  Total $-1,426.44.  All point to account 10.3810.</t>
+        </is>
+      </c>
+      <c r="C34" s="96" t="n"/>
+      <c r="D34" s="96" t="n"/>
+      <c r="E34" s="96" t="n"/>
+    </row>
+    <row r="35" ht="112" customHeight="1" s="29">
+      <c r="A35" s="97" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="B35" s="98" t="inlineStr">
+        <is>
+          <t>These batches are fully approved and just need R09801 to run for Company 00010.  This is normal end-of-period activity — inventory transactions entered late on the last day of the period accumulate at "Approved / Approved" status until the next scheduled posting run.
+No batch-by-batch action is needed.  No approval action is needed.  The count of 8 batches from a single user on a single account on consecutive days suggests routine inventory entry, not a problem.</t>
+        </is>
+      </c>
+      <c r="C35" s="99" t="n"/>
+      <c r="D35" s="99" t="n"/>
+      <c r="E35" s="99" t="n"/>
+    </row>
+    <row r="36" ht="96" customHeight="1" s="29">
+      <c r="A36" s="94" t="inlineStr">
+        <is>
+          <t>Resolution</t>
+        </is>
+      </c>
+      <c r="B36" s="95" t="inlineStr">
+        <is>
+          <t>Step 1.  Run R09801 for Company 00010.  All 8 approved N-type batches will be posted in the run.
+Step 2.  After the run completes, refresh RapidReconciler and confirm Company 00010 GL Batches variance has decreased by $1,426.44.
+Step 3.  If any of these 8 batches remain unposted after R09801 runs, investigate as a posting error (Section 9 of the GL Batch guide).</t>
+        </is>
+      </c>
+      <c r="C36" s="96" t="n"/>
+      <c r="D36" s="96" t="n"/>
+      <c r="E36" s="96" t="n"/>
+    </row>
+    <row r="37" ht="10" customHeight="1" s="29"/>
+    <row r="38" ht="28" customHeight="1" s="29">
+      <c r="A38" s="82" t="inlineStr">
+        <is>
+          <t>Action Plan  (in execution order)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1" s="29">
+      <c r="A39" s="102" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B39" s="103" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C50" s="45" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="154" customHeight="1" s="29">
-      <c r="A51" s="58" t="inlineStr">
-        <is>
-          <t>1 — URGENT</t>
-        </is>
-      </c>
-      <c r="B51" s="22" t="inlineStr">
-        <is>
-          <t>Open the Batch Header Revisions screen (P0011) in JD Edwards for each of the five O-type batches (7000001, 7000002, 7000004, 7000005, 7000006) in Co 00080. For each batch, manually set the posting status to blank (unposted). Approve each batch, then run R09801 to post. Engage IT to investigate why the SCHED01 scheduler posting is being interrupted for O-type batches in Co 00080 — the 29-day age of the oldest batch indicates this is a recurring issue. Configure alerting so future occurrences are caught immediately.</t>
-        </is>
-      </c>
-      <c r="C51" s="59" t="inlineStr">
-        <is>
-          <t>IT / Finance</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="70" customHeight="1" s="29">
-      <c r="A52" s="43" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B52" s="24" t="inlineStr">
-        <is>
-          <t>Review and approve IB batch 7000003 (USER01, Co 00090). Both account rows (90010.3810 and 90040.3810) are part of the same batch — review the inventory balance adjustment before approving. Run R09801 after approval.</t>
-        </is>
-      </c>
-      <c r="C52" s="60" t="inlineStr">
-        <is>
-          <t>Finance / USER01</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="56" customHeight="1" s="29">
-      <c r="A53" s="58" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B53" s="22" t="inlineStr">
-        <is>
-          <t>Review and approve G batch 7000007 (USER02, Co 00070, $-767.40). This is a manual journal entry — confirm with USER02 the purpose and obtain supervisor sign-off per policy. Run R09801 after approval.</t>
-        </is>
-      </c>
-      <c r="C53" s="59" t="inlineStr">
-        <is>
-          <t>Finance Supervisor</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="56" customHeight="1" s="29">
-      <c r="A54" s="43" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B54" s="24" t="inlineStr">
-        <is>
-          <t>Review and approve V batch 7000008 (USER04, Co 00030, $13,354.12). Confirm the AP voucher is valid and the supplier invoice matches. Run R09801 after approval.</t>
-        </is>
-      </c>
-      <c r="C54" s="60" t="inlineStr">
+      <c r="E39" s="103" t="inlineStr">
+        <is>
+          <t>Owner / Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="64" customHeight="1" s="29">
+      <c r="A40" s="104" t="n">
+        <v>1</v>
+      </c>
+      <c r="B40" s="95" t="inlineStr">
+        <is>
+          <t>Reset and post the 5 "In Use" O-type batches in Co 80 (Finding 1).  In P0011, set posting status back to blank for each batch, approve, then run R09801.  Largest dollar impact ($156,598.12); oldest is 29 days old.</t>
+        </is>
+      </c>
+      <c r="C40" s="96" t="n"/>
+      <c r="D40" s="96" t="n"/>
+      <c r="E40" s="105" t="inlineStr">
+        <is>
+          <t>Finance / IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="64" customHeight="1" s="29">
+      <c r="A41" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="98" t="inlineStr">
+        <is>
+          <t>Engage IT to investigate the SCHED01 receipt-posting failure (Finding 1 root cause).  This is recurring — without alerting, new "In Use" batches will accumulate.  Configure scheduler alerting before the next period.</t>
+        </is>
+      </c>
+      <c r="C41" s="99" t="n"/>
+      <c r="D41" s="99" t="n"/>
+      <c r="E41" s="107" t="inlineStr">
+        <is>
+          <t>IT Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="64" customHeight="1" s="29">
+      <c r="A42" s="104" t="n">
+        <v>3</v>
+      </c>
+      <c r="B42" s="95" t="inlineStr">
+        <is>
+          <t>Review and approve IB batch 7000003 in Co 90 (Finding 2).  Both account rows must be approved together.  Verify the adjustment makes accounting sense before approving — contact USER01 if anything looks off.</t>
+        </is>
+      </c>
+      <c r="C42" s="96" t="n"/>
+      <c r="D42" s="96" t="n"/>
+      <c r="E42" s="105" t="inlineStr">
+        <is>
+          <t>Inventory Accounting / USER01</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="50" customHeight="1" s="29">
+      <c r="A43" s="106" t="n">
+        <v>4</v>
+      </c>
+      <c r="B43" s="98" t="inlineStr">
+        <is>
+          <t>Review and approve V batch 7000008 in Co 30 (Finding 4).  Verify the supplier invoice matches and the GL account is correct for the purchase.</t>
+        </is>
+      </c>
+      <c r="C43" s="99" t="n"/>
+      <c r="D43" s="99" t="n"/>
+      <c r="E43" s="107" t="inlineStr">
         <is>
           <t>AP / USER04</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="42" customHeight="1" s="29">
-      <c r="A55" s="58" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B55" s="22" t="inlineStr">
-        <is>
-          <t>Run R09801 for Co 00010 to post all 8 approved N-type batches (USER03). No approval action required — batches are already approved.</t>
-        </is>
-      </c>
-      <c r="C55" s="59" t="inlineStr">
+    <row r="44" ht="64" customHeight="1" s="29">
+      <c r="A44" s="104" t="n">
+        <v>5</v>
+      </c>
+      <c r="B44" s="95" t="inlineStr">
+        <is>
+          <t>Review and approve G batch 7000007 in Co 70 (Finding 3).  Manual journal entry — confirm purpose with USER02 and obtain supervisor sign-off per segregation-of-duties policy.</t>
+        </is>
+      </c>
+      <c r="C44" s="96" t="n"/>
+      <c r="D44" s="96" t="n"/>
+      <c r="E44" s="105" t="inlineStr">
+        <is>
+          <t>Finance Supervisor / USER02</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="50" customHeight="1" s="29">
+      <c r="A45" s="106" t="n">
+        <v>6</v>
+      </c>
+      <c r="B45" s="98" t="inlineStr">
+        <is>
+          <t>Run R09801 for Co 10 to post the 8 approved N-type batches (Finding 5).  No approval action required — routine.</t>
+        </is>
+      </c>
+      <c r="C45" s="99" t="n"/>
+      <c r="D45" s="99" t="n"/>
+      <c r="E45" s="107" t="inlineStr">
         <is>
           <t>Finance / IT</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="70" customHeight="1" s="29">
-      <c r="A56" s="43" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B56" s="24" t="inlineStr">
-        <is>
-          <t>After all batches are posted, confirm the GL Batches variance in RapidReconciler = $0 for the March 2026 period. If any residual balance remains, check for additional unposted batches or run R099102 to repost account balances.</t>
-        </is>
-      </c>
-      <c r="C56" s="60" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="16" customHeight="1" s="29">
-      <c r="A57" s="41" t="n"/>
-      <c r="B57" s="41" t="n"/>
-      <c r="C57" s="41" t="n"/>
-    </row>
-    <row r="58" ht="42" customHeight="1" s="29">
-      <c r="A58" s="61" t="inlineStr">
-        <is>
-          <t>Analysis generated by Claude — April 22, 2026</t>
+    <row r="46" ht="80" customHeight="1" s="29">
+      <c r="A46" s="104" t="n">
+        <v>7</v>
+      </c>
+      <c r="B46" s="95" t="inlineStr">
+        <is>
+          <t>Period-close gate: do not post closing journal entries until GL Batches variance is $0.  Confirm via RapidReconciler refresh after each posting run.  If any residual remains, run R099102 to repost account balances or check for additional unposted batches.</t>
+        </is>
+      </c>
+      <c r="C46" s="96" t="n"/>
+      <c r="D46" s="96" t="n"/>
+      <c r="E46" s="105" t="inlineStr">
+        <is>
+          <t>Finance / Controller</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="14" customHeight="1" s="29"/>
+    <row r="48" ht="70" customHeight="1" s="29">
+      <c r="A48" s="108" t="inlineStr">
+        <is>
+          <t>⚠  Before approving any batch in P0011:  verify the underlying transaction is correct (supplier invoice, journal purpose, account assignment).  Approving an incorrectly entered batch will post bad data to F0902 — much harder to fix than a pre-approval correction.  Do not post period-close journal entries until GL Batches variance is $0.</t>
+        </is>
+      </c>
+      <c r="B48" s="109" t="n"/>
+      <c r="C48" s="109" t="n"/>
+      <c r="D48" s="109" t="n"/>
+      <c r="E48" s="109" t="n"/>
+    </row>
+    <row r="49" ht="8" customHeight="1" s="29"/>
+    <row r="50" ht="18" customHeight="1" s="29">
+      <c r="A50" s="110" t="inlineStr">
+        <is>
+          <t>Analysis produced using the Unposted GL Batches Report Guide  ·  RapidReconciler  ·  April 25, 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A49:C49"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A58:C58"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="A26:C26"/>
+  <mergeCells count="49">
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A35"/>
+    <mergeCell ref="A29"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="A20"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="A19"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="A31"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="A34"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="A30"/>
+    <mergeCell ref="A15"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="A24"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="A36"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="A25"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A16"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A26"/>
+    <mergeCell ref="A21"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="A14"/>
+    <mergeCell ref="B34:E34"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId100"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2978,7 +3112,7 @@
       <c r="M19" s="74" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:M2"/>
+  <autoFilter ref="A2:M19"/>
   <mergeCells count="1">
     <mergeCell ref="A1:M1"/>
   </mergeCells>

</xml_diff>